<commit_message>
added some essences #1
</commit_message>
<xml_diff>
--- a/draft/database_eft.xlsx
+++ b/draft/database_eft.xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="182">
-  <si>
-    <t>quest</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="235">
+  <si>
+    <t xml:space="preserve">  </t>
   </si>
   <si>
     <t>таблица со всеми квестами</t>
@@ -439,12 +439,12 @@
     <t>up_level</t>
   </si>
   <si>
-    <t>TODO... таблица бартера</t>
-  </si>
-  <si>
     <t>kill_zryachy</t>
   </si>
   <si>
+    <t>min_fence_loyalty</t>
+  </si>
+  <si>
     <t>map</t>
   </si>
   <si>
@@ -469,12 +469,21 @@
     <t>таблица ценами продажи торговцев</t>
   </si>
   <si>
+    <t>items_barter</t>
+  </si>
+  <si>
+    <t>таблица с бартером</t>
+  </si>
+  <si>
     <t>image</t>
   </si>
   <si>
     <t>max_pmc</t>
   </si>
   <si>
+    <t>unlock_flea_market</t>
+  </si>
+  <si>
     <t>trader</t>
   </si>
   <si>
@@ -484,6 +493,9 @@
     <t>valuta</t>
   </si>
   <si>
+    <t>max_count</t>
+  </si>
+  <si>
     <t>Название карты</t>
   </si>
   <si>
@@ -502,6 +514,9 @@
     <t>тип предмета</t>
   </si>
   <si>
+    <t>с какого уровня доступен на барахолке</t>
+  </si>
+  <si>
     <t>ID предложения</t>
   </si>
   <si>
@@ -517,6 +532,12 @@
     <t>цена продажи</t>
   </si>
   <si>
+    <t>сколько можно купить за 1 завоз</t>
+  </si>
+  <si>
+    <t>количество</t>
+  </si>
+  <si>
     <t>Избыточно будет если сделать ID как уникальный ключ</t>
   </si>
   <si>
@@ -529,6 +550,9 @@
     <t>у каждой категории предметов есть свои категории свойств (как у бутылки воды может быть 1.42 MOA?)</t>
   </si>
   <si>
+    <t>вот чем и грешат старые справочники. До релиза было просто: барахолка доступна только с уровня N, и она давала доступ абсолютно ко всем предметам. Теперь же мало того, что не каждый предмет доступен на барахолке, так еще и становится доступен с уровня N. Можно было привязать доступность к категории предмета, но некоторые предметы -- исключение из правил. Например, ключи можно покупать только с 25 уровня, но ключи от "меченок" доступны с 35 уровня, а танковый аккум хоть и относится к категории электроника (доступен с 20 уровня), но доступен с 40 уровня. Если поле на записи здесь пустое, значит предмет не доступен на барахолке, потому что сама барахолка открывается с 15 уровня</t>
+  </si>
+  <si>
     <t>поскольку один и тот же предмет могут купить разные торговцы за разную стоимость, поэтому идея "1 item = 1 item_purchase" не подходит. Если цены нет, значит торговец не покупает</t>
   </si>
   <si>
@@ -541,10 +565,7 @@
     <t>да, пока тогровцы скупают за рубль, кроме миротворца, однако судя по развитию игры, а также по наличию других валют, лучше сделать этот пункт</t>
   </si>
   <si>
-    <t>аналогично с itmes_purchase</t>
-  </si>
-  <si>
-    <t>тот, кто продает этот предмет</t>
+    <t>тот, кто продает этот предмет. Указываем по уровню лояльности</t>
   </si>
   <si>
     <t>то, за сколько продает торговец</t>
@@ -553,17 +574,155 @@
     <t>здесь проще, чем в items_purchase, потому что торговцы часто продают по разнообразной валюте</t>
   </si>
   <si>
+    <t>можно было бы привязать ID предложения к ID item, но торговец имеет наглость просить за 1 предмет несколько разных предметов</t>
+  </si>
+  <si>
+    <t>кто предлагает. Указываем по уровню лояльности</t>
+  </si>
+  <si>
+    <t>торговец может требовать за 1 предмет несколько разных, но правильней говорить несколько категорий предметов. Например, Миротворец 2LL требует за защищенный кейс Бета 1 танковый аккум, 5 военных кабелей, 3 виртекса и 3 иридиума</t>
+  </si>
+  <si>
     <t>text not null primary key</t>
   </si>
   <si>
     <t>text</t>
+  </si>
+  <si>
+    <t>TODO... описать каждую категорию</t>
+  </si>
+  <si>
+    <t>TODO... создать сущность, описывающая свойства из этой категории</t>
+  </si>
+  <si>
+    <t>bladed_weapons</t>
+  </si>
+  <si>
+    <t>weapons</t>
+  </si>
+  <si>
+    <t>bullets</t>
+  </si>
+  <si>
+    <t>mods</t>
+  </si>
+  <si>
+    <t>specs</t>
+  </si>
+  <si>
+    <t>food</t>
+  </si>
+  <si>
+    <t>medicine</t>
+  </si>
+  <si>
+    <t>containers</t>
+  </si>
+  <si>
+    <t>keys</t>
+  </si>
+  <si>
+    <t>armors</t>
+  </si>
+  <si>
+    <t>таблица с торговцами</t>
+  </si>
+  <si>
+    <t>trader_loyalty</t>
+  </si>
+  <si>
+    <t>таблица хранящая информацию о лояльности торговцев</t>
+  </si>
+  <si>
+    <t>items_unlocking_purchase</t>
+  </si>
+  <si>
+    <t>таблица с доступными предметами к покупке после квеста</t>
+  </si>
+  <si>
+    <t>in_raid</t>
+  </si>
+  <si>
+    <t>trader_name</t>
+  </si>
+  <si>
+    <t>loyalty_level</t>
+  </si>
+  <si>
+    <t>min_loyalty</t>
+  </si>
+  <si>
+    <t>min_turnover_amount</t>
+  </si>
+  <si>
+    <t>unlocked_in_quest</t>
+  </si>
+  <si>
+    <t>имя торговца</t>
+  </si>
+  <si>
+    <t>иконка торговца</t>
+  </si>
+  <si>
+    <t>встретить только в рейде</t>
+  </si>
+  <si>
+    <t>уровень лояльности</t>
+  </si>
+  <si>
+    <t>с каким торговцем связан LL</t>
+  </si>
+  <si>
+    <t>минимальный уровень</t>
+  </si>
+  <si>
+    <t>минимальная лояльность</t>
+  </si>
+  <si>
+    <t>минимальный оборот средств</t>
+  </si>
+  <si>
+    <t>нужно ли открывать по квесту</t>
+  </si>
+  <si>
+    <t>с каким квестом связан</t>
+  </si>
+  <si>
+    <t>торговцев немного, поэтому их имена можно использовать в качестве PK</t>
+  </si>
+  <si>
+    <t>да, смотрителя и водителя БТР сложно назвать торговцами, но они выдают квесты, а также на будущее будет запас, вдруг они не только будут выдавать квесты и оказывать услуги</t>
+  </si>
+  <si>
+    <t>опишем как id, чтобы удобнее было условия разблокировки. Благо условия разблокировки простые, нужно открыть за выполнение квестов, а повышать по простой схеме: min_level AND min_loyalty AND min_turnover_amount</t>
+  </si>
+  <si>
+    <t>проблема в том, что есть 3 типа торговцев: классическая LL (1..3 и prime), упрощенная (у скупщика, 1 и prime) и вообще без репутации (ни на что не влияет, записей о них здесь делать не нужно)</t>
+  </si>
+  <si>
+    <t>тут просто, уровней 1..3 и prime, для простоты назовем prime LL просто 4</t>
+  </si>
+  <si>
+    <t>если уровень не нужен, то просто 0</t>
+  </si>
+  <si>
+    <t>если не нужен, то просто 0</t>
+  </si>
+  <si>
+    <t>да, не все торговцы доступны сразу по 1LL, некоторых нужно открывать по сюжетному квесту "Тур", либо выполняя какой-то побочный квест (Легкие деньги часть 1 на Рефа LL1, Поручение на Егеря LL1 и Новое знакомство на Смотрителя)</t>
+  </si>
+  <si>
+    <t>берем с таблицы лояльности</t>
+  </si>
+  <si>
+    <t>какой квест разблокировывает бартер</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -594,6 +753,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -758,7 +923,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="48">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -801,6 +966,7 @@
     <xf borderId="9" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="5" fontId="1" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="10" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -834,18 +1000,27 @@
     <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="10" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="10" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="14" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="14" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="5" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="7" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
@@ -858,8 +1033,12 @@
     <xf borderId="10" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
+    <xf borderId="12" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="7" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="14" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="7" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -867,13 +1046,18 @@
     <xf borderId="10" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="0" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1095,26 +1279,29 @@
     <col customWidth="1" min="2" max="2" width="32.5"/>
     <col customWidth="1" min="3" max="3" width="30.0"/>
     <col customWidth="1" min="4" max="4" width="19.38"/>
-    <col customWidth="1" min="5" max="6" width="20.13"/>
+    <col customWidth="1" min="5" max="5" width="32.25"/>
+    <col customWidth="1" min="6" max="6" width="29.0"/>
     <col customWidth="1" min="7" max="7" width="20.63"/>
     <col customWidth="1" min="8" max="8" width="31.5"/>
-    <col customWidth="1" min="9" max="9" width="20.25"/>
-    <col customWidth="1" min="10" max="10" width="27.63"/>
-    <col customWidth="1" min="11" max="11" width="19.13"/>
+    <col customWidth="1" min="9" max="9" width="22.88"/>
+    <col customWidth="1" min="10" max="10" width="62.88"/>
+    <col customWidth="1" min="11" max="11" width="34.5"/>
     <col customWidth="1" min="12" max="12" width="24.25"/>
     <col customWidth="1" min="13" max="13" width="21.88"/>
     <col customWidth="1" min="14" max="14" width="19.75"/>
     <col customWidth="1" min="15" max="15" width="25.25"/>
     <col customWidth="1" min="16" max="16" width="20.13"/>
-    <col customWidth="1" min="17" max="17" width="21.88"/>
+    <col customWidth="1" min="17" max="17" width="26.38"/>
     <col customWidth="1" min="18" max="18" width="22.88"/>
     <col customWidth="1" min="19" max="19" width="18.63"/>
     <col customWidth="1" min="20" max="20" width="31.88"/>
     <col customWidth="1" min="21" max="21" width="30.25"/>
-    <col customWidth="1" min="22" max="23" width="23.5"/>
-    <col customWidth="1" min="24" max="24" width="13.88"/>
+    <col customWidth="1" min="22" max="22" width="23.5"/>
+    <col customWidth="1" min="23" max="23" width="28.25"/>
+    <col customWidth="1" min="24" max="24" width="26.38"/>
     <col customWidth="1" min="25" max="25" width="18.88"/>
-    <col customWidth="1" min="26" max="26" width="63.63"/>
+    <col customWidth="1" min="26" max="26" width="62.88"/>
+    <col customWidth="1" min="27" max="28" width="31.88"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1257,6 +1444,8 @@
       <c r="T3" s="15" t="s">
         <v>38</v>
       </c>
+      <c r="AA3" s="16"/>
+      <c r="AB3" s="16"/>
     </row>
     <row r="4">
       <c r="A4" s="12" t="s">
@@ -1310,74 +1499,80 @@
       <c r="T4" s="15" t="s">
         <v>49</v>
       </c>
+      <c r="AA4" s="16"/>
+      <c r="AB4" s="16"/>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="H5" s="18" t="s">
+      <c r="H5" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="I5" s="16" t="s">
+      <c r="I5" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="J5" s="16" t="s">
+      <c r="J5" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="L5" s="16" t="s">
+      <c r="L5" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="M5" s="16" t="s">
+      <c r="M5" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="N5" s="16" t="s">
+      <c r="N5" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="O5" s="16" t="s">
+      <c r="O5" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="P5" s="16" t="s">
+      <c r="P5" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="R5" s="18" t="s">
+      <c r="R5" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="S5" s="19" t="s">
+      <c r="S5" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="T5" s="20" t="s">
+      <c r="T5" s="21" t="s">
         <v>55</v>
       </c>
+      <c r="AA5" s="16"/>
+      <c r="AB5" s="16"/>
     </row>
     <row r="6">
-      <c r="A6" s="21"/>
-      <c r="H6" s="21"/>
+      <c r="A6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="AA6" s="16"/>
+      <c r="AB6" s="16"/>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="23" t="s">
+      <c r="B7" s="24" t="s">
         <v>57</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="4"/>
-      <c r="F7" s="24" t="s">
+      <c r="F7" s="25" t="s">
         <v>58</v>
       </c>
       <c r="G7" s="8" t="s">
@@ -1387,7 +1582,7 @@
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="4"/>
-      <c r="M7" s="25" t="s">
+      <c r="M7" s="26" t="s">
         <v>60</v>
       </c>
       <c r="N7" s="8" t="s">
@@ -1408,9 +1603,11 @@
       <c r="Y7" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="Z7" s="26" t="s">
+      <c r="Z7" s="27" t="s">
         <v>65</v>
       </c>
+      <c r="AA7" s="28"/>
+      <c r="AB7" s="28"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="s">
@@ -1428,19 +1625,19 @@
       <c r="F8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G8" s="27" t="s">
+      <c r="G8" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="H8" s="27" t="s">
+      <c r="H8" s="29" t="s">
         <v>70</v>
       </c>
-      <c r="I8" s="28" t="s">
+      <c r="I8" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="J8" s="28" t="s">
+      <c r="J8" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="K8" s="28" t="s">
+      <c r="K8" s="30" t="s">
         <v>11</v>
       </c>
       <c r="M8" s="7" t="s">
@@ -1479,6 +1676,8 @@
       <c r="Z8" s="9" t="s">
         <v>75</v>
       </c>
+      <c r="AA8" s="31"/>
+      <c r="AB8" s="31"/>
     </row>
     <row r="9">
       <c r="A9" s="12" t="s">
@@ -1547,6 +1746,8 @@
       <c r="Z9" s="12" t="s">
         <v>93</v>
       </c>
+      <c r="AA9" s="31"/>
+      <c r="AB9" s="31"/>
     </row>
     <row r="10">
       <c r="A10" s="12" t="s">
@@ -1615,551 +1816,938 @@
       <c r="Z10" s="12" t="s">
         <v>39</v>
       </c>
+      <c r="AA10" s="31"/>
+      <c r="AB10" s="31"/>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="F11" s="16" t="s">
+      <c r="F11" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="G11" s="16" t="s">
+      <c r="G11" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="H11" s="16" t="s">
+      <c r="H11" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="I11" s="16" t="s">
+      <c r="I11" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="J11" s="16" t="s">
+      <c r="J11" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="K11" s="16" t="s">
+      <c r="K11" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="M11" s="16" t="s">
+      <c r="M11" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="N11" s="16" t="s">
+      <c r="N11" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="O11" s="16" t="s">
+      <c r="O11" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="P11" s="16" t="s">
+      <c r="P11" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="Q11" s="16" t="s">
+      <c r="Q11" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="R11" s="16" t="s">
+      <c r="R11" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="T11" s="16" t="s">
+      <c r="T11" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="U11" s="16" t="s">
+      <c r="U11" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="V11" s="16" t="s">
+      <c r="V11" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="W11" s="16" t="s">
+      <c r="W11" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="Y11" s="16" t="s">
+      <c r="Y11" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="Z11" s="16" t="s">
+      <c r="Z11" s="17" t="s">
         <v>51</v>
       </c>
+      <c r="AA11" s="31"/>
+      <c r="AB11" s="31"/>
     </row>
     <row r="12">
-      <c r="C12" s="29" t="s">
+      <c r="C12" s="32" t="s">
         <v>112</v>
       </c>
-      <c r="J12" s="30" t="s">
+      <c r="J12" s="33" t="s">
         <v>113</v>
       </c>
-      <c r="O12" s="30" t="s">
+      <c r="O12" s="33" t="s">
         <v>114</v>
       </c>
-      <c r="V12" s="30" t="s">
+      <c r="V12" s="33" t="s">
         <v>115</v>
       </c>
-      <c r="Z12" s="30" t="s">
+      <c r="Z12" s="33" t="s">
         <v>116</v>
       </c>
+      <c r="AA12" s="34"/>
+      <c r="AB12" s="34"/>
     </row>
     <row r="13">
-      <c r="C13" s="31" t="s">
+      <c r="C13" s="35" t="s">
         <v>117</v>
       </c>
-      <c r="J13" s="32" t="s">
+      <c r="J13" s="36" t="s">
         <v>118</v>
       </c>
-      <c r="O13" s="32" t="s">
+      <c r="O13" s="36" t="s">
         <v>119</v>
       </c>
-      <c r="V13" s="32" t="s">
+      <c r="V13" s="36" t="s">
         <v>120</v>
       </c>
-      <c r="Z13" s="32" t="s">
+      <c r="Z13" s="36" t="s">
         <v>121</v>
       </c>
+      <c r="AA13" s="34"/>
+      <c r="AB13" s="34"/>
     </row>
     <row r="14">
-      <c r="C14" s="31" t="s">
+      <c r="C14" s="35" t="s">
         <v>122</v>
       </c>
-      <c r="J14" s="32" t="s">
+      <c r="J14" s="36" t="s">
         <v>123</v>
       </c>
-      <c r="O14" s="32" t="s">
+      <c r="O14" s="36" t="s">
         <v>124</v>
       </c>
-      <c r="V14" s="32" t="s">
+      <c r="V14" s="36" t="s">
         <v>125</v>
       </c>
-      <c r="Z14" s="33" t="s">
+      <c r="Z14" s="37" t="s">
         <v>120</v>
       </c>
+      <c r="AA14" s="34"/>
+      <c r="AB14" s="34"/>
     </row>
     <row r="15">
-      <c r="C15" s="31" t="s">
+      <c r="C15" s="35" t="s">
         <v>126</v>
       </c>
-      <c r="J15" s="32" t="s">
+      <c r="J15" s="36" t="s">
         <v>127</v>
       </c>
-      <c r="O15" s="32" t="s">
+      <c r="O15" s="36" t="s">
         <v>128</v>
       </c>
-      <c r="V15" s="33" t="s">
+      <c r="V15" s="37" t="s">
         <v>129</v>
       </c>
+      <c r="AA15" s="16"/>
+      <c r="AB15" s="16"/>
     </row>
     <row r="16">
-      <c r="C16" s="31" t="s">
+      <c r="C16" s="35" t="s">
         <v>130</v>
       </c>
-      <c r="J16" s="32" t="s">
+      <c r="J16" s="36" t="s">
         <v>131</v>
       </c>
-      <c r="O16" s="32" t="s">
+      <c r="O16" s="36" t="s">
         <v>132</v>
       </c>
+      <c r="AA16" s="16"/>
+      <c r="AB16" s="16"/>
     </row>
     <row r="17">
-      <c r="C17" s="31" t="s">
+      <c r="C17" s="35" t="s">
         <v>133</v>
       </c>
-      <c r="J17" s="32" t="s">
+      <c r="J17" s="36" t="s">
         <v>134</v>
       </c>
-      <c r="O17" s="32" t="s">
+      <c r="O17" s="36" t="s">
         <v>135</v>
       </c>
+      <c r="AA17" s="16"/>
+      <c r="AB17" s="16"/>
     </row>
     <row r="18">
-      <c r="C18" s="31" t="s">
+      <c r="C18" s="35" t="s">
         <v>136</v>
       </c>
-      <c r="J18" s="33" t="s">
+      <c r="J18" s="37" t="s">
         <v>137</v>
       </c>
-      <c r="O18" s="32" t="s">
+      <c r="O18" s="36" t="s">
         <v>138</v>
       </c>
+      <c r="AA18" s="16"/>
+      <c r="AB18" s="16"/>
     </row>
     <row r="19">
-      <c r="C19" s="31" t="s">
+      <c r="C19" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="O19" s="32" t="s">
+      <c r="O19" s="36" t="s">
         <v>139</v>
       </c>
+      <c r="AA19" s="16"/>
+      <c r="AB19" s="16"/>
     </row>
     <row r="20">
-      <c r="C20" s="31" t="s">
+      <c r="C20" s="35" t="s">
         <v>140</v>
       </c>
-      <c r="O20" s="33" t="s">
+      <c r="O20" s="37" t="s">
         <v>141</v>
       </c>
-      <c r="R20" s="21" t="s">
+      <c r="AA20" s="16"/>
+      <c r="AB20" s="16"/>
+    </row>
+    <row r="21">
+      <c r="C21" s="35" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="21">
-      <c r="C21" s="34" t="s">
+      <c r="AA21" s="16"/>
+      <c r="AB21" s="16"/>
+    </row>
+    <row r="22">
+      <c r="C22" s="38" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="22">
-      <c r="C22" s="35"/>
+      <c r="AA22" s="16"/>
+      <c r="AB22" s="16"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="C23" s="4"/>
-      <c r="E23" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="4"/>
-      <c r="K23" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="L23" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="M23" s="3"/>
-      <c r="N23" s="3"/>
-      <c r="O23" s="4"/>
-      <c r="Q23" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="R23" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="S23" s="3"/>
-      <c r="T23" s="3"/>
-      <c r="U23" s="4"/>
+      <c r="AB23" s="39"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="C24" s="4"/>
+      <c r="E24" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="4"/>
+      <c r="L24" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="M24" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="N24" s="3"/>
+      <c r="O24" s="3"/>
+      <c r="P24" s="4"/>
+      <c r="R24" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="S24" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="T24" s="3"/>
+      <c r="U24" s="3"/>
+      <c r="V24" s="3"/>
+      <c r="W24" s="4"/>
+      <c r="Y24" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="Z24" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="AA24" s="3"/>
+      <c r="AB24" s="4"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B24" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="E24" s="7" t="s">
+      <c r="B25" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="E25" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F25" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="G24" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="H24" s="7" t="s">
+      <c r="G25" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="H25" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="I24" s="7" t="s">
+      <c r="I25" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="K24" s="7" t="s">
+      <c r="J25" s="40" t="s">
+        <v>156</v>
+      </c>
+      <c r="L25" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="L24" s="7" t="s">
+      <c r="M25" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="M24" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="N24" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="O24" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="Q24" s="7" t="s">
+      <c r="N25" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="O25" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="P25" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="R25" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="R24" s="7" t="s">
+      <c r="S25" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="S24" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="T24" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="U24" s="7" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="12" t="s">
+      <c r="T25" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="U25" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="C25" s="12" t="s">
+      <c r="V25" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="E25" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="F25" s="12" t="s">
+      <c r="W25" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="G25" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="H25" s="12" t="s">
-        <v>162</v>
-      </c>
-      <c r="I25" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="K25" s="12" t="s">
-        <v>163</v>
-      </c>
-      <c r="L25" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="M25" s="12" t="s">
-        <v>164</v>
-      </c>
-      <c r="N25" s="12" t="s">
-        <v>165</v>
-      </c>
-      <c r="O25" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="Q25" s="12" t="s">
-        <v>163</v>
-      </c>
-      <c r="R25" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="S25" s="12" t="s">
-        <v>164</v>
-      </c>
-      <c r="T25" s="12" t="s">
-        <v>167</v>
-      </c>
-      <c r="U25" s="12" t="s">
-        <v>166</v>
+      <c r="Y25" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="Z25" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="AA25" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="AB25" s="7" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="H26" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="I26" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="J26" s="41" t="s">
+        <v>167</v>
+      </c>
+      <c r="L26" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="B26" s="36" t="s">
+      <c r="M26" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="N26" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="C26" s="12" t="s">
+      <c r="O26" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="P26" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="R26" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="S26" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="T26" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="U26" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="V26" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="W26" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="Y26" s="41" t="s">
+        <v>168</v>
+      </c>
+      <c r="Z26" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA26" s="41" t="s">
+        <v>169</v>
+      </c>
+      <c r="AB26" s="41" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="B27" s="42" t="s">
+        <v>176</v>
+      </c>
+      <c r="C27" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="E26" s="12" t="s">
+      <c r="E27" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="F26" s="12" t="s">
+      <c r="F27" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="G26" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="H26" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="I26" s="12" t="s">
+      <c r="G27" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="H27" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="I27" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="K26" s="12" t="s">
+      <c r="J27" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="L27" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="L26" s="12" t="s">
-        <v>172</v>
-      </c>
-      <c r="M26" s="12" t="s">
+      <c r="M27" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="N27" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="O27" s="12" t="s">
+        <v>182</v>
+      </c>
+      <c r="P27" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="R27" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="S27" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="T27" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="U27" s="12" t="s">
+        <v>185</v>
+      </c>
+      <c r="V27" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="W27" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y27" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="Z27" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="AA27" s="12" t="s">
+        <v>188</v>
+      </c>
+      <c r="AB27" s="12" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="B28" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="C28" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="E28" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="F28" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="G28" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="H28" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="I28" s="17" t="s">
+        <v>191</v>
+      </c>
+      <c r="J28" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="L28" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="M28" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="N28" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="O28" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="P28" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="R28" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="S28" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="T28" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="U28" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="V28" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="W28" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="Y28" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="Z28" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA28" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB28" s="17" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="31"/>
+      <c r="B29" s="44"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="31"/>
+      <c r="G29" s="31"/>
+      <c r="H29" s="31" t="s">
+        <v>192</v>
+      </c>
+      <c r="I29" s="31"/>
+      <c r="L29" s="22"/>
+      <c r="M29" s="22"/>
+      <c r="N29" s="22"/>
+      <c r="O29" s="22"/>
+      <c r="P29" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="V29" s="33" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="31"/>
+      <c r="B30" s="44"/>
+      <c r="C30" s="31"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="31"/>
+      <c r="G30" s="31"/>
+      <c r="H30" s="31" t="s">
+        <v>193</v>
+      </c>
+      <c r="I30" s="31"/>
+      <c r="L30" s="22"/>
+      <c r="M30" s="22"/>
+      <c r="N30" s="22"/>
+      <c r="O30" s="22"/>
+      <c r="P30" s="36" t="s">
+        <v>124</v>
+      </c>
+      <c r="V30" s="36" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="31"/>
+      <c r="B31" s="44"/>
+      <c r="C31" s="31"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="31" t="s">
+        <v>194</v>
+      </c>
+      <c r="F31" s="31" t="s">
+        <v>195</v>
+      </c>
+      <c r="G31" s="31" t="s">
+        <v>196</v>
+      </c>
+      <c r="H31" s="31" t="s">
+        <v>197</v>
+      </c>
+      <c r="I31" s="31" t="s">
+        <v>198</v>
+      </c>
+      <c r="J31" s="22" t="s">
+        <v>199</v>
+      </c>
+      <c r="L31" s="22"/>
+      <c r="M31" s="22"/>
+      <c r="N31" s="22"/>
+      <c r="O31" s="22"/>
+      <c r="P31" s="36" t="s">
+        <v>128</v>
+      </c>
+      <c r="V31" s="36" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="31"/>
+      <c r="B32" s="44"/>
+      <c r="C32" s="31"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="31" t="s">
+        <v>200</v>
+      </c>
+      <c r="F32" s="31" t="s">
+        <v>201</v>
+      </c>
+      <c r="G32" s="31" t="s">
+        <v>202</v>
+      </c>
+      <c r="H32" s="31" t="s">
+        <v>203</v>
+      </c>
+      <c r="I32" s="31"/>
+      <c r="L32" s="22"/>
+      <c r="M32" s="22"/>
+      <c r="N32" s="22"/>
+      <c r="O32" s="22"/>
+      <c r="P32" s="37" t="s">
+        <v>132</v>
+      </c>
+      <c r="V32" s="37" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="31"/>
+      <c r="B33" s="44"/>
+      <c r="C33" s="31"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="31"/>
+      <c r="F33" s="31"/>
+      <c r="G33" s="31"/>
+      <c r="H33" s="31"/>
+      <c r="I33" s="31"/>
+      <c r="K33" s="22"/>
+      <c r="L33" s="22"/>
+      <c r="M33" s="22"/>
+      <c r="N33" s="22"/>
+      <c r="O33" s="45"/>
+      <c r="U33" s="45"/>
+      <c r="AA33" s="16"/>
+      <c r="AB33" s="16"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="B34" s="46" t="s">
+        <v>204</v>
+      </c>
+      <c r="C34" s="4"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="3"/>
+      <c r="K34" s="4"/>
+      <c r="L34" s="22"/>
+      <c r="M34" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="N34" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="O34" s="3"/>
+      <c r="P34" s="3"/>
+      <c r="Q34" s="4"/>
+      <c r="U34" s="45"/>
+      <c r="AA34" s="16"/>
+      <c r="AB34" s="16"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B35" s="47" t="s">
+        <v>154</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="D35" s="16"/>
+      <c r="E35" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="G35" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="H35" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="I35" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="J35" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="K35" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="L35" s="22"/>
+      <c r="M35" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="N35" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="O35" s="47" t="s">
+        <v>157</v>
+      </c>
+      <c r="P35" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q35" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="U35" s="45"/>
+      <c r="AA35" s="16"/>
+      <c r="AB35" s="16"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="B36" s="42" t="s">
+        <v>216</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="D36" s="16"/>
+      <c r="E36" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="F36" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="G36" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="H36" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="I36" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="J36" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="K36" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="L36" s="22"/>
+      <c r="M36" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="N36" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="O36" s="42" t="s">
+        <v>169</v>
+      </c>
+      <c r="P36" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="Q36" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="N26" s="12" t="s">
-        <v>174</v>
-      </c>
-      <c r="O26" s="12" t="s">
-        <v>175</v>
-      </c>
-      <c r="Q26" s="12" t="s">
+      <c r="U36" s="45"/>
+      <c r="AA36" s="16"/>
+      <c r="AB36" s="16"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="s">
+        <v>225</v>
+      </c>
+      <c r="B37" s="42" t="s">
+        <v>177</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="D37" s="16"/>
+      <c r="E37" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="F37" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="G37" s="12" t="s">
+        <v>229</v>
+      </c>
+      <c r="H37" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="I37" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="J37" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="K37" s="12" t="s">
+        <v>232</v>
+      </c>
+      <c r="L37" s="22"/>
+      <c r="M37" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="R26" s="12" t="s">
-        <v>176</v>
-      </c>
-      <c r="S26" s="12" t="s">
-        <v>177</v>
-      </c>
-      <c r="T26" s="12" t="s">
-        <v>178</v>
-      </c>
-      <c r="U26" s="12" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="16" t="s">
-        <v>180</v>
-      </c>
-      <c r="B27" s="37" t="s">
+      <c r="N37" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="O37" s="42" t="s">
+        <v>233</v>
+      </c>
+      <c r="P37" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="Q37" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="U37" s="45"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="B38" s="43" t="s">
         <v>51</v>
       </c>
-      <c r="C27" s="16" t="s">
+      <c r="C38" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="D38" s="16"/>
+      <c r="E38" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="F38" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="G38" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="E27" s="16" t="s">
+      <c r="H38" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="I38" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="J38" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="K38" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="L38" s="22"/>
+      <c r="M38" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="F27" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="G27" s="16" t="s">
-        <v>180</v>
-      </c>
-      <c r="H27" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="I27" s="16" t="s">
-        <v>181</v>
-      </c>
-      <c r="K27" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="L27" s="16" t="s">
+      <c r="N38" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="M27" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="N27" s="16" t="s">
+      <c r="O38" s="43" t="s">
         <v>53</v>
       </c>
-      <c r="O27" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q27" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="R27" s="16" t="s">
+      <c r="P38" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="S27" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="T27" s="16" t="s">
+      <c r="Q38" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="U27" s="16" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="38"/>
-      <c r="B28" s="39"/>
-      <c r="C28" s="38"/>
-      <c r="D28" s="40"/>
-      <c r="E28" s="38"/>
-      <c r="F28" s="38"/>
-      <c r="G28" s="38"/>
-      <c r="H28" s="38"/>
-      <c r="I28" s="38"/>
-      <c r="K28" s="21"/>
-      <c r="L28" s="21"/>
-      <c r="M28" s="21"/>
-      <c r="N28" s="21"/>
-      <c r="O28" s="30" t="s">
-        <v>119</v>
-      </c>
-      <c r="U28" s="30" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="38"/>
-      <c r="B29" s="39"/>
-      <c r="C29" s="38"/>
-      <c r="D29" s="40"/>
-      <c r="E29" s="38"/>
-      <c r="F29" s="38"/>
-      <c r="G29" s="38"/>
-      <c r="H29" s="38"/>
-      <c r="I29" s="38"/>
-      <c r="K29" s="21"/>
-      <c r="L29" s="21"/>
-      <c r="M29" s="21"/>
-      <c r="N29" s="21"/>
-      <c r="O29" s="32" t="s">
-        <v>124</v>
-      </c>
-      <c r="U29" s="32" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="38"/>
-      <c r="B30" s="39"/>
-      <c r="C30" s="38"/>
-      <c r="D30" s="40"/>
-      <c r="E30" s="38"/>
-      <c r="F30" s="38"/>
-      <c r="G30" s="38"/>
-      <c r="H30" s="38"/>
-      <c r="I30" s="38"/>
-      <c r="K30" s="21"/>
-      <c r="L30" s="21"/>
-      <c r="M30" s="21"/>
-      <c r="N30" s="21"/>
-      <c r="O30" s="32" t="s">
-        <v>128</v>
-      </c>
-      <c r="U30" s="32" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="38"/>
-      <c r="B31" s="39"/>
-      <c r="C31" s="38"/>
-      <c r="D31" s="40"/>
-      <c r="E31" s="38"/>
-      <c r="F31" s="38"/>
-      <c r="G31" s="38"/>
-      <c r="H31" s="38"/>
-      <c r="I31" s="38"/>
-      <c r="K31" s="21"/>
-      <c r="L31" s="21"/>
-      <c r="M31" s="21"/>
-      <c r="N31" s="21"/>
-      <c r="O31" s="33" t="s">
-        <v>132</v>
-      </c>
-      <c r="U31" s="33" t="s">
-        <v>132</v>
-      </c>
+      <c r="U38" s="45"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="F23:I23"/>
-    <mergeCell ref="L23:O23"/>
-    <mergeCell ref="R23:U23"/>
+  <mergeCells count="16">
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="I1:J1"/>
     <mergeCell ref="M1:P1"/>
@@ -2167,6 +2755,15 @@
     <mergeCell ref="G7:K7"/>
     <mergeCell ref="N7:R7"/>
     <mergeCell ref="U7:W7"/>
+    <mergeCell ref="F34:K34"/>
+    <mergeCell ref="N34:Q34"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="F24:J24"/>
+    <mergeCell ref="M24:P24"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="S24:W24"/>
+    <mergeCell ref="Z24:AB24"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>